<commit_message>
Mahal listesine sıhhi tesisat eklendi (MAHAL-SIHHI-PROFORMA)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/05_MAHAL_LISTESI.xlsx
+++ b/belgeler/05_MAHAL_LISTESI.xlsx
@@ -652,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1705,76 +1705,249 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Sıhhi Tesisat</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C35" s="37" t="inlineStr">
+        <is>
+          <t>Temiz su tesisatı — PPRC boru ve ek parçaları, küresel vanalar, askı ve kılıflar</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E35" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F35" s="38" t="inlineStr"/>
+      <c r="G35" s="38" t="inlineStr"/>
+      <c r="H35" s="38" t="inlineStr"/>
+      <c r="I35" s="38" t="inlineStr"/>
+      <c r="J35" s="38" t="inlineStr"/>
+      <c r="K35" s="38" t="inlineStr"/>
+      <c r="L35" s="38" t="inlineStr"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="14" t="n"/>
+      <c r="B36" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C36" s="37" t="inlineStr">
+        <is>
+          <t>Pis su tesisatı — Ø50 / Ø70 / Ø100 sert PVC boru, temizleme kapağı, yer süzgeci</t>
+        </is>
+      </c>
+      <c r="D36" s="38" t="inlineStr"/>
+      <c r="E36" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F36" s="38" t="inlineStr"/>
+      <c r="G36" s="38" t="inlineStr"/>
+      <c r="H36" s="38" t="inlineStr"/>
+      <c r="I36" s="38" t="inlineStr"/>
+      <c r="J36" s="38" t="inlineStr"/>
+      <c r="K36" s="38" t="inlineStr"/>
+      <c r="L36" s="38" t="inlineStr"/>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="14" t="n"/>
+      <c r="B37" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C37" s="37" t="inlineStr">
+        <is>
+          <t>Termosifon — sıcak su üretimi</t>
+        </is>
+      </c>
+      <c r="D37" s="38" t="inlineStr"/>
+      <c r="E37" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F37" s="38" t="inlineStr"/>
+      <c r="G37" s="38" t="inlineStr"/>
+      <c r="H37" s="38" t="inlineStr"/>
+      <c r="I37" s="38" t="inlineStr"/>
+      <c r="J37" s="38" t="inlineStr"/>
+      <c r="K37" s="38" t="inlineStr"/>
+      <c r="L37" s="38" t="inlineStr"/>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="14" t="n"/>
+      <c r="B38" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C38" s="37" t="inlineStr">
+        <is>
+          <t>Şebeke su bağlantısı ve 2" su sayacı</t>
+        </is>
+      </c>
+      <c r="D38" s="38" t="inlineStr"/>
+      <c r="E38" s="38" t="inlineStr"/>
+      <c r="F38" s="38" t="inlineStr"/>
+      <c r="G38" s="38" t="inlineStr"/>
+      <c r="H38" s="38" t="inlineStr"/>
+      <c r="I38" s="38" t="inlineStr"/>
+      <c r="J38" s="38" t="inlineStr"/>
+      <c r="K38" s="38" t="inlineStr"/>
+      <c r="L38" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="14" t="n"/>
+      <c r="B39" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C39" s="37" t="inlineStr">
+        <is>
+          <t>Hidrofor — Q = 2 m³/h, P = 33-38 mSS</t>
+        </is>
+      </c>
+      <c r="D39" s="38" t="inlineStr"/>
+      <c r="E39" s="38" t="inlineStr"/>
+      <c r="F39" s="38" t="inlineStr"/>
+      <c r="G39" s="38" t="inlineStr"/>
+      <c r="H39" s="38" t="inlineStr"/>
+      <c r="I39" s="38" t="inlineStr"/>
+      <c r="J39" s="38" t="inlineStr"/>
+      <c r="K39" s="38" t="inlineStr"/>
+      <c r="L39" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="15" t="n"/>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C40" s="37" t="inlineStr">
+        <is>
+          <t>Tesisat hidroforu — 0,3 m³/h, 30 mSS</t>
+        </is>
+      </c>
+      <c r="D40" s="38" t="inlineStr"/>
+      <c r="E40" s="38" t="inlineStr"/>
+      <c r="F40" s="38" t="inlineStr"/>
+      <c r="G40" s="38" t="inlineStr"/>
+      <c r="H40" s="38" t="inlineStr"/>
+      <c r="I40" s="38" t="inlineStr"/>
+      <c r="J40" s="38" t="inlineStr"/>
+      <c r="K40" s="38" t="inlineStr"/>
+      <c r="L40" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t>AÇIKLAMALAR</t>
         </is>
       </c>
-      <c r="B36" s="40" t="n"/>
-      <c r="C36" s="40" t="n"/>
-      <c r="D36" s="40" t="n"/>
-      <c r="E36" s="40" t="n"/>
-      <c r="F36" s="40" t="n"/>
-      <c r="G36" s="40" t="n"/>
-      <c r="H36" s="40" t="n"/>
-      <c r="I36" s="40" t="n"/>
-      <c r="J36" s="40" t="n"/>
-      <c r="K36" s="40" t="n"/>
-      <c r="L36" s="41" t="n"/>
-    </row>
-    <row r="37" ht="13" customHeight="1">
-      <c r="A37" s="17" t="inlineStr">
+      <c r="B42" s="40" t="n"/>
+      <c r="C42" s="40" t="n"/>
+      <c r="D42" s="40" t="n"/>
+      <c r="E42" s="40" t="n"/>
+      <c r="F42" s="40" t="n"/>
+      <c r="G42" s="40" t="n"/>
+      <c r="H42" s="40" t="n"/>
+      <c r="I42" s="40" t="n"/>
+      <c r="J42" s="40" t="n"/>
+      <c r="K42" s="40" t="n"/>
+      <c r="L42" s="41" t="n"/>
+    </row>
+    <row r="43" ht="13" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>•  Mahal listesi, mimari projenin ekinde sunulmak üzere hazırlanmıştır; mahal kodları mimari plandaki blok ve hacim adlarıyla eşleşir.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="13" customHeight="1">
-      <c r="A38" s="17" t="inlineStr">
+    <row r="44" ht="13" customHeight="1">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>•  Listede kullanılan poz numaraları metraj cetveli ve keşif özetiyle birebir aynıdır.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="13" customHeight="1">
-      <c r="A39" s="17" t="inlineStr">
+    <row r="45" ht="13" customHeight="1">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>•  Kümes A ve B blok birebir özdeş olduğundan tek mahal sütununda gösterilmiştir.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="17" t="inlineStr">
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>•  Listedeki pozların tamamı birim fiyat kitaplarındandır: 15.xxx ÇŞB 2026 birim fiyat kitabı, TKDK-xxxx ise TKDK 17.02.2026 Özel Poz Tablosu pozudur.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="17" t="inlineStr">
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>•  Sıhhi tesisat kalemlerinin kitap pozu yoktur ve keşif özetinde yer almazlar: miktarları onaylı sıhhi tesisat projesinden, bedelleri piyasa araştırmasından gelir ve 36 numaralı proforma ile beyan edilir. Poz sütununda “—” işareti bunu gösterir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>•  Gübre çukuru, ölü atma çukuru ve depoların iç yüzeyleri kaplamasız brüt betonarmedir; su yalıtımı bu hesabın kapsamı dışında bırakılmıştır. Foseptik betonarme değildir: kazı ve grobeton oturma yatağı üzerine yerleştirilen prefabrik polietilen sızdırmaz tanktır.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="A38:L38"/>
+  <mergeCells count="18">
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A35:A40"/>
+    <mergeCell ref="A42:L42"/>
     <mergeCell ref="A22:A23"/>
-    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="A43:L43"/>
     <mergeCell ref="A24:A27"/>
+    <mergeCell ref="A47:L47"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A28:A30"/>
-    <mergeCell ref="A37:L37"/>
-    <mergeCell ref="A36:L36"/>
+    <mergeCell ref="A45:L45"/>
+    <mergeCell ref="A46:L46"/>
     <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A40:L40"/>
+    <mergeCell ref="A44:L44"/>
     <mergeCell ref="A14:A21"/>
     <mergeCell ref="A31:A33"/>
     <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A39:L39"/>
+    <mergeCell ref="A48:L48"/>
     <mergeCell ref="A6:A10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>